<commit_message>
add prototype code has added.
</commit_message>
<xml_diff>
--- a/02.機能設計/端子割り当て.xlsx
+++ b/02.機能設計/端子割り当て.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/872dd85359dadb48/OneDrive/技術検討/raspberry Pi pico debug/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\01_Software\RaspiPico\DialKeyPad\02.機能設計\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="323" documentId="11_AD4D066CA252ABDACC10481E5950E8FA73EEDF5D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BD0CF2E-83F5-40EF-97D5-E0C6BC226A94}"/>
   <bookViews>
-    <workbookView xWindow="5265" yWindow="5220" windowWidth="29520" windowHeight="15780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8040" yWindow="3000" windowWidth="21060" windowHeight="15780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="端子一覧" sheetId="1" r:id="rId1"/>
@@ -3444,7 +3444,7 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="1">
-        <f t="shared" ref="B7:B55" si="0">B6+1</f>
+        <f t="shared" ref="B7:B44" si="0">B6+1</f>
         <v>3</v>
       </c>
       <c r="C7" s="3" t="s">

</xml_diff>